<commit_message>
code updates, 2025 spreadsheet
</commit_message>
<xml_diff>
--- a/spreadsheets/CSD_codes/CSD_codes.xlsx
+++ b/spreadsheets/CSD_codes/CSD_codes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/ward_1792_osu_edu/Documents/brooke_BLD/Beech-Leaf-Disease-/data/BLD_county_level/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/ward_1792_osu_edu/Documents/_research/ohio_state/beech_leaf_disease/beech_leaf_disease_spread/beech_leaf_disease_laptop/spreadsheets/CSD_codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="8_{4BD1E2E8-3ACD-4E3A-BD13-2446748DB92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08942330-C46A-4BDA-9A8F-8F6D8E53820D}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="8_{4BD1E2E8-3ACD-4E3A-BD13-2446748DB92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A625FAFE-F201-4879-8DA9-3F351E58D7FE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F614C848-5D6D-4E14-8EA7-0A5C31DBA8E5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F614C848-5D6D-4E14-8EA7-0A5C31DBA8E5}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>Census division</t>
   </si>
@@ -559,6 +559,87 @@
   </si>
   <si>
     <t>Chatahm Kent</t>
+  </si>
+  <si>
+    <t>Dufferin</t>
+  </si>
+  <si>
+    <t>Bruce</t>
+  </si>
+  <si>
+    <t>Grey</t>
+  </si>
+  <si>
+    <t>Haliburton</t>
+  </si>
+  <si>
+    <t>Renfrew</t>
+  </si>
+  <si>
+    <t>Nipissing</t>
+  </si>
+  <si>
+    <t>Muskoka District</t>
+  </si>
+  <si>
+    <t>Parry Sound</t>
+  </si>
+  <si>
+    <t>Manitoulin</t>
+  </si>
+  <si>
+    <t>Sudbury</t>
+  </si>
+  <si>
+    <t>Kenora</t>
+  </si>
+  <si>
+    <t>Rainy River</t>
+  </si>
+  <si>
+    <t>Thunder Bay</t>
+  </si>
+  <si>
+    <t>Algoma</t>
+  </si>
+  <si>
+    <t>Cochrane</t>
+  </si>
+  <si>
+    <t>Timiskaming</t>
+  </si>
+  <si>
+    <t>Greater Sudbury</t>
+  </si>
+  <si>
+    <t>York</t>
+  </si>
+  <si>
+    <t>Kawartha Lakes</t>
+  </si>
+  <si>
+    <t>Prince Edward</t>
+  </si>
+  <si>
+    <t>Lennox and Addington</t>
+  </si>
+  <si>
+    <t>Frontenac</t>
+  </si>
+  <si>
+    <t>Lanark</t>
+  </si>
+  <si>
+    <t>Leeds and Grenville United</t>
+  </si>
+  <si>
+    <t>Ottawa</t>
+  </si>
+  <si>
+    <t>Prescott and Russell United</t>
+  </si>
+  <si>
+    <t>Stormont, Dundas and Glengarry United</t>
   </si>
 </sst>
 </file>
@@ -611,10 +692,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -967,6 +1044,9 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
+      <c r="D2" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -978,6 +1058,9 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
+      <c r="D3" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -989,6 +1072,9 @@
       <c r="C4" t="s">
         <v>6</v>
       </c>
+      <c r="D4" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1000,6 +1086,9 @@
       <c r="C5" t="s">
         <v>8</v>
       </c>
+      <c r="D5" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1011,6 +1100,9 @@
       <c r="C6" t="s">
         <v>10</v>
       </c>
+      <c r="D6" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1022,6 +1114,9 @@
       <c r="C7" t="s">
         <v>12</v>
       </c>
+      <c r="D7" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1033,6 +1128,9 @@
       <c r="C8" t="s">
         <v>14</v>
       </c>
+      <c r="D8" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1058,6 +1156,9 @@
       <c r="C10" t="s">
         <v>18</v>
       </c>
+      <c r="D10" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1097,6 +1198,9 @@
       <c r="C13" t="s">
         <v>24</v>
       </c>
+      <c r="D13" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1122,6 +1226,9 @@
       <c r="C15" t="s">
         <v>28</v>
       </c>
+      <c r="D15" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1161,6 +1268,9 @@
       <c r="C18" t="s">
         <v>34</v>
       </c>
+      <c r="D18" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1382,6 +1492,9 @@
       <c r="C34" t="s">
         <v>66</v>
       </c>
+      <c r="D34" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
@@ -1393,6 +1506,9 @@
       <c r="C35" t="s">
         <v>68</v>
       </c>
+      <c r="D35" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
@@ -1418,6 +1534,9 @@
       <c r="C37" t="s">
         <v>72</v>
       </c>
+      <c r="D37" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
@@ -1429,6 +1548,9 @@
       <c r="C38" t="s">
         <v>74</v>
       </c>
+      <c r="D38" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
@@ -1440,6 +1562,9 @@
       <c r="C39" t="s">
         <v>76</v>
       </c>
+      <c r="D39" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
@@ -1451,6 +1576,9 @@
       <c r="C40" t="s">
         <v>78</v>
       </c>
+      <c r="D40" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
@@ -1462,6 +1590,9 @@
       <c r="C41" t="s">
         <v>80</v>
       </c>
+      <c r="D41" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
@@ -1473,6 +1604,9 @@
       <c r="C42" t="s">
         <v>82</v>
       </c>
+      <c r="D42" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
@@ -1484,6 +1618,9 @@
       <c r="C43" t="s">
         <v>84</v>
       </c>
+      <c r="D43" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
@@ -1495,6 +1632,9 @@
       <c r="C44" t="s">
         <v>86</v>
       </c>
+      <c r="D44" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
@@ -1506,6 +1646,9 @@
       <c r="C45" t="s">
         <v>88</v>
       </c>
+      <c r="D45" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
@@ -1517,6 +1660,9 @@
       <c r="C46" t="s">
         <v>90</v>
       </c>
+      <c r="D46" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
@@ -1528,6 +1674,9 @@
       <c r="C47" t="s">
         <v>92</v>
       </c>
+      <c r="D47" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
@@ -1539,8 +1688,11 @@
       <c r="C48" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D48" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>147</v>
       </c>
@@ -1550,8 +1702,11 @@
       <c r="C49" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>148</v>
       </c>
@@ -1560,6 +1715,9 @@
       </c>
       <c r="C50" t="s">
         <v>98</v>
+      </c>
+      <c r="D50" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>